<commit_message>
feat(mcp): add account remediation use cases
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/tutorials/mcp/mcp_sqlite_excel/data/account_review_dataset.xlsx
+++ b/tutorials/mcp/mcp_sqlite_excel/data/account_review_dataset.xlsx
@@ -553,7 +553,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AI16"/>
+  <dimension ref="A1:CS16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -598,7 +598,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -773,6 +772,316 @@
       <c r="AI4" t="inlineStr">
         <is>
           <t>CRD Number</t>
+        </is>
+      </c>
+      <c r="AJ4" t="inlineStr">
+        <is>
+          <t>Action Owner</t>
+        </is>
+      </c>
+      <c r="AK4" t="inlineStr">
+        <is>
+          <t>Action Title</t>
+        </is>
+      </c>
+      <c r="AL4" t="inlineStr">
+        <is>
+          <t>Action Explanation</t>
+        </is>
+      </c>
+      <c r="AM4" t="inlineStr">
+        <is>
+          <t>Action Button</t>
+        </is>
+      </c>
+      <c r="AN4" t="inlineStr">
+        <is>
+          <t>Action Button Target</t>
+        </is>
+      </c>
+      <c r="AO4" t="inlineStr">
+        <is>
+          <t>Fig1 Label</t>
+        </is>
+      </c>
+      <c r="AP4" t="inlineStr">
+        <is>
+          <t>Fig1 Value</t>
+        </is>
+      </c>
+      <c r="AQ4" t="inlineStr">
+        <is>
+          <t>Fig1 Status</t>
+        </is>
+      </c>
+      <c r="AR4" t="inlineStr">
+        <is>
+          <t>Fig1 Pct</t>
+        </is>
+      </c>
+      <c r="AS4" t="inlineStr">
+        <is>
+          <t>Fig2 Label</t>
+        </is>
+      </c>
+      <c r="AT4" t="inlineStr">
+        <is>
+          <t>Fig2 Value</t>
+        </is>
+      </c>
+      <c r="AU4" t="inlineStr">
+        <is>
+          <t>Fig2 Status</t>
+        </is>
+      </c>
+      <c r="AV4" t="inlineStr">
+        <is>
+          <t>Fig2 Pct</t>
+        </is>
+      </c>
+      <c r="AW4" t="inlineStr">
+        <is>
+          <t>Fig3 Label</t>
+        </is>
+      </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>Fig3 Value</t>
+        </is>
+      </c>
+      <c r="AY4" t="inlineStr">
+        <is>
+          <t>Fig3 Status</t>
+        </is>
+      </c>
+      <c r="AZ4" t="inlineStr">
+        <is>
+          <t>Fig3 Pct</t>
+        </is>
+      </c>
+      <c r="BA4" t="inlineStr">
+        <is>
+          <t>Perf1 Label</t>
+        </is>
+      </c>
+      <c r="BB4" t="inlineStr">
+        <is>
+          <t>Perf1 Value</t>
+        </is>
+      </c>
+      <c r="BC4" t="inlineStr">
+        <is>
+          <t>Perf1 Status</t>
+        </is>
+      </c>
+      <c r="BD4" t="inlineStr">
+        <is>
+          <t>Perf1 Pct</t>
+        </is>
+      </c>
+      <c r="BE4" t="inlineStr">
+        <is>
+          <t>Perf2 Label</t>
+        </is>
+      </c>
+      <c r="BF4" t="inlineStr">
+        <is>
+          <t>Perf2 Value</t>
+        </is>
+      </c>
+      <c r="BG4" t="inlineStr">
+        <is>
+          <t>Perf2 Status</t>
+        </is>
+      </c>
+      <c r="BH4" t="inlineStr">
+        <is>
+          <t>Perf2 Pct</t>
+        </is>
+      </c>
+      <c r="BI4" t="inlineStr">
+        <is>
+          <t>Perf3 Label</t>
+        </is>
+      </c>
+      <c r="BJ4" t="inlineStr">
+        <is>
+          <t>Perf3 Value</t>
+        </is>
+      </c>
+      <c r="BK4" t="inlineStr">
+        <is>
+          <t>Perf3 Status</t>
+        </is>
+      </c>
+      <c r="BL4" t="inlineStr">
+        <is>
+          <t>Perf3 Pct</t>
+        </is>
+      </c>
+      <c r="BM4" s="3" t="inlineStr">
+        <is>
+          <t>Mandate Type</t>
+        </is>
+      </c>
+      <c r="BN4" s="3" t="inlineStr">
+        <is>
+          <t>Mand1 Label</t>
+        </is>
+      </c>
+      <c r="BO4" s="3" t="inlineStr">
+        <is>
+          <t>Mand1 Value</t>
+        </is>
+      </c>
+      <c r="BP4" s="3" t="inlineStr">
+        <is>
+          <t>Mand1 Status</t>
+        </is>
+      </c>
+      <c r="BQ4" s="3" t="inlineStr">
+        <is>
+          <t>Mand1 Pct</t>
+        </is>
+      </c>
+      <c r="BR4" s="3" t="inlineStr">
+        <is>
+          <t>Mand2 Label</t>
+        </is>
+      </c>
+      <c r="BS4" s="3" t="inlineStr">
+        <is>
+          <t>Mand2 Value</t>
+        </is>
+      </c>
+      <c r="BT4" s="3" t="inlineStr">
+        <is>
+          <t>Mand2 Status</t>
+        </is>
+      </c>
+      <c r="BU4" s="3" t="inlineStr">
+        <is>
+          <t>Mand2 Pct</t>
+        </is>
+      </c>
+      <c r="BV4" s="3" t="inlineStr">
+        <is>
+          <t>Mand3 Label</t>
+        </is>
+      </c>
+      <c r="BW4" s="3" t="inlineStr">
+        <is>
+          <t>Mand3 Value</t>
+        </is>
+      </c>
+      <c r="BX4" s="3" t="inlineStr">
+        <is>
+          <t>Mand3 Status</t>
+        </is>
+      </c>
+      <c r="BY4" s="3" t="inlineStr">
+        <is>
+          <t>Mand3 Pct</t>
+        </is>
+      </c>
+      <c r="BZ4" s="3" t="inlineStr">
+        <is>
+          <t>Client Categorization</t>
+        </is>
+      </c>
+      <c r="CA4" s="3" t="inlineStr">
+        <is>
+          <t>Category Required</t>
+        </is>
+      </c>
+      <c r="CB4" s="3" t="inlineStr">
+        <is>
+          <t>Category Review Status</t>
+        </is>
+      </c>
+      <c r="CC4" s="3" t="inlineStr">
+        <is>
+          <t>Hold1 Label</t>
+        </is>
+      </c>
+      <c r="CD4" s="3" t="inlineStr">
+        <is>
+          <t>Hold1 Value</t>
+        </is>
+      </c>
+      <c r="CE4" s="3" t="inlineStr">
+        <is>
+          <t>Hold1 Status</t>
+        </is>
+      </c>
+      <c r="CF4" s="3" t="inlineStr">
+        <is>
+          <t>Hold1 Pct</t>
+        </is>
+      </c>
+      <c r="CG4" s="3" t="inlineStr">
+        <is>
+          <t>Hold2 Label</t>
+        </is>
+      </c>
+      <c r="CH4" s="3" t="inlineStr">
+        <is>
+          <t>Hold2 Value</t>
+        </is>
+      </c>
+      <c r="CI4" s="3" t="inlineStr">
+        <is>
+          <t>Hold2 Status</t>
+        </is>
+      </c>
+      <c r="CJ4" s="3" t="inlineStr">
+        <is>
+          <t>Hold2 Pct</t>
+        </is>
+      </c>
+      <c r="CK4" s="3" t="inlineStr">
+        <is>
+          <t>Hold3 Label</t>
+        </is>
+      </c>
+      <c r="CL4" s="3" t="inlineStr">
+        <is>
+          <t>Hold3 Value</t>
+        </is>
+      </c>
+      <c r="CM4" s="3" t="inlineStr">
+        <is>
+          <t>Hold3 Status</t>
+        </is>
+      </c>
+      <c r="CN4" s="3" t="inlineStr">
+        <is>
+          <t>Hold3 Pct</t>
+        </is>
+      </c>
+      <c r="CO4" s="3" t="inlineStr">
+        <is>
+          <t>Risk Tolerance</t>
+        </is>
+      </c>
+      <c r="CP4" s="3" t="inlineStr">
+        <is>
+          <t>Investment Horizon</t>
+        </is>
+      </c>
+      <c r="CQ4" s="3" t="inlineStr">
+        <is>
+          <t>Knowledge Experience</t>
+        </is>
+      </c>
+      <c r="CR4" s="3" t="inlineStr">
+        <is>
+          <t>Last Suitability Test</t>
+        </is>
+      </c>
+      <c r="CS4" s="3" t="inlineStr">
+        <is>
+          <t>Suitability Outcome</t>
         </is>
       </c>
     </row>
@@ -946,6 +1255,274 @@
           <t>CRD-CH-0187</t>
         </is>
       </c>
+      <c r="AJ5" t="inlineStr">
+        <is>
+          <t>Compliance</t>
+        </is>
+      </c>
+      <c r="AK5" t="inlineStr">
+        <is>
+          <t>Adverse media — escalated to Compliance</t>
+        </is>
+      </c>
+      <c r="AL5" t="inlineStr">
+        <is>
+          <t>WorldCheck flagged adverse media relating to ongoing litigation. Case has been escalated; the client has been given the opportunity to comment before Compliance resolves it.</t>
+        </is>
+      </c>
+      <c r="AM5" t="inlineStr">
+        <is>
+          <t>View case file</t>
+        </is>
+      </c>
+      <c r="AN5" t="inlineStr">
+        <is>
+          <t>cont_case_CH-priv-0187</t>
+        </is>
+      </c>
+      <c r="AO5" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="AP5" t="inlineStr">
+        <is>
+          <t>WorldCheck</t>
+        </is>
+      </c>
+      <c r="AQ5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AS5" t="inlineStr">
+        <is>
+          <t>Match</t>
+        </is>
+      </c>
+      <c r="AT5" t="inlineStr">
+        <is>
+          <t>Adverse media — ongoing litigation</t>
+        </is>
+      </c>
+      <c r="AU5" t="inlineStr">
+        <is>
+          <t>warn</t>
+        </is>
+      </c>
+      <c r="AW5" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="AX5" t="inlineStr">
+        <is>
+          <t>With Compliance — client comment pending</t>
+        </is>
+      </c>
+      <c r="AY5" t="inlineStr">
+        <is>
+          <t>warn</t>
+        </is>
+      </c>
+      <c r="BA5" t="inlineStr">
+        <is>
+          <t>Portfolio return (YTD)</t>
+        </is>
+      </c>
+      <c r="BB5" t="inlineStr">
+        <is>
+          <t>+9.2%</t>
+        </is>
+      </c>
+      <c r="BC5" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="BE5" t="inlineStr">
+        <is>
+          <t>Benchmark — MSCI ACWI</t>
+        </is>
+      </c>
+      <c r="BF5" t="inlineStr">
+        <is>
+          <t>+8.4%</t>
+        </is>
+      </c>
+      <c r="BG5" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="BI5" t="inlineStr">
+        <is>
+          <t>Variance vs benchmark</t>
+        </is>
+      </c>
+      <c r="BJ5" t="inlineStr">
+        <is>
+          <t>+0.8 pp</t>
+        </is>
+      </c>
+      <c r="BK5" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="BM5" t="inlineStr">
+        <is>
+          <t>Discretionary — Growth</t>
+        </is>
+      </c>
+      <c r="BN5" t="inlineStr">
+        <is>
+          <t>Equity</t>
+        </is>
+      </c>
+      <c r="BO5" t="inlineStr">
+        <is>
+          <t>66% (ceiling 75%)</t>
+        </is>
+      </c>
+      <c r="BP5" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="BQ5" t="n">
+        <v>66</v>
+      </c>
+      <c r="BR5" t="inlineStr">
+        <is>
+          <t>Fixed income</t>
+        </is>
+      </c>
+      <c r="BS5" t="inlineStr">
+        <is>
+          <t>22% (band ≤30%)</t>
+        </is>
+      </c>
+      <c r="BT5" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="BU5" t="n">
+        <v>22</v>
+      </c>
+      <c r="BV5" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="BW5" t="inlineStr">
+        <is>
+          <t>12% (band ≥5%)</t>
+        </is>
+      </c>
+      <c r="BX5" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="BY5" t="n">
+        <v>12</v>
+      </c>
+      <c r="BZ5" t="inlineStr">
+        <is>
+          <t>Professional client (per-se)</t>
+        </is>
+      </c>
+      <c r="CA5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CB5" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="CC5" t="inlineStr">
+        <is>
+          <t>Equities — Global Large Cap</t>
+        </is>
+      </c>
+      <c r="CD5" t="inlineStr">
+        <is>
+          <t>38%</t>
+        </is>
+      </c>
+      <c r="CE5" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="CF5" t="n">
+        <v>38</v>
+      </c>
+      <c r="CG5" t="inlineStr">
+        <is>
+          <t>Private Equity / Alternatives</t>
+        </is>
+      </c>
+      <c r="CH5" t="inlineStr">
+        <is>
+          <t>24%</t>
+        </is>
+      </c>
+      <c r="CI5" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="CJ5" t="n">
+        <v>24</v>
+      </c>
+      <c r="CK5" t="inlineStr">
+        <is>
+          <t>Fixed Income — EM Corporate</t>
+        </is>
+      </c>
+      <c r="CL5" t="inlineStr">
+        <is>
+          <t>18%</t>
+        </is>
+      </c>
+      <c r="CM5" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="CN5" t="n">
+        <v>18</v>
+      </c>
+      <c r="CO5" t="inlineStr">
+        <is>
+          <t>Growth</t>
+        </is>
+      </c>
+      <c r="CP5" t="inlineStr">
+        <is>
+          <t>10+ years</t>
+        </is>
+      </c>
+      <c r="CQ5" t="inlineStr">
+        <is>
+          <t>Advanced — active trader</t>
+        </is>
+      </c>
+      <c r="CR5" t="inlineStr">
+        <is>
+          <t>2026-03-02</t>
+        </is>
+      </c>
+      <c r="CS5" t="inlineStr">
+        <is>
+          <t>Aligned with Growth mandate</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -1117,6 +1694,274 @@
           <t>CRD-CH-0204</t>
         </is>
       </c>
+      <c r="AJ6" t="inlineStr">
+        <is>
+          <t>Compliance</t>
+        </is>
+      </c>
+      <c r="AK6" t="inlineStr">
+        <is>
+          <t>PEP — enhanced due diligence refresh</t>
+        </is>
+      </c>
+      <c r="AL6" t="inlineStr">
+        <is>
+          <t>Client is a politically exposed person; the periodic EDD pack is being refreshed by Compliance as part of ongoing monitoring.</t>
+        </is>
+      </c>
+      <c r="AM6" t="inlineStr">
+        <is>
+          <t>View EDD status</t>
+        </is>
+      </c>
+      <c r="AN6" t="inlineStr">
+        <is>
+          <t>cont_edd_CH-priv-0204</t>
+        </is>
+      </c>
+      <c r="AO6" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="AP6" t="inlineStr">
+        <is>
+          <t>WorldCheck</t>
+        </is>
+      </c>
+      <c r="AQ6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AS6" t="inlineStr">
+        <is>
+          <t>Match</t>
+        </is>
+      </c>
+      <c r="AT6" t="inlineStr">
+        <is>
+          <t>PEP status — EDD refresh</t>
+        </is>
+      </c>
+      <c r="AU6" t="inlineStr">
+        <is>
+          <t>warn</t>
+        </is>
+      </c>
+      <c r="AW6" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>With Compliance — EDD in progress</t>
+        </is>
+      </c>
+      <c r="AY6" t="inlineStr">
+        <is>
+          <t>warn</t>
+        </is>
+      </c>
+      <c r="BA6" t="inlineStr">
+        <is>
+          <t>Portfolio return (YTD)</t>
+        </is>
+      </c>
+      <c r="BB6" t="inlineStr">
+        <is>
+          <t>+5.6%</t>
+        </is>
+      </c>
+      <c r="BC6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="BE6" t="inlineStr">
+        <is>
+          <t>Benchmark — 60/40 blended</t>
+        </is>
+      </c>
+      <c r="BF6" t="inlineStr">
+        <is>
+          <t>+6.1%</t>
+        </is>
+      </c>
+      <c r="BG6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="BI6" t="inlineStr">
+        <is>
+          <t>Variance vs benchmark</t>
+        </is>
+      </c>
+      <c r="BJ6" t="inlineStr">
+        <is>
+          <t>-0.5 pp</t>
+        </is>
+      </c>
+      <c r="BK6" t="inlineStr">
+        <is>
+          <t>warn</t>
+        </is>
+      </c>
+      <c r="BM6" t="inlineStr">
+        <is>
+          <t>Discretionary — Balanced</t>
+        </is>
+      </c>
+      <c r="BN6" t="inlineStr">
+        <is>
+          <t>Equity</t>
+        </is>
+      </c>
+      <c r="BO6" t="inlineStr">
+        <is>
+          <t>48% (ceiling 60%)</t>
+        </is>
+      </c>
+      <c r="BP6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="BQ6" t="n">
+        <v>48</v>
+      </c>
+      <c r="BR6" t="inlineStr">
+        <is>
+          <t>Fixed income</t>
+        </is>
+      </c>
+      <c r="BS6" t="inlineStr">
+        <is>
+          <t>38% (band ≤45%)</t>
+        </is>
+      </c>
+      <c r="BT6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="BU6" t="n">
+        <v>38</v>
+      </c>
+      <c r="BV6" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="BW6" t="inlineStr">
+        <is>
+          <t>14% (band ≥5%)</t>
+        </is>
+      </c>
+      <c r="BX6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="BY6" t="n">
+        <v>14</v>
+      </c>
+      <c r="BZ6" t="inlineStr">
+        <is>
+          <t>Retail — MiFID standard</t>
+        </is>
+      </c>
+      <c r="CA6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CB6" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="CC6" t="inlineStr">
+        <is>
+          <t>Fixed Income — UK Gilts</t>
+        </is>
+      </c>
+      <c r="CD6" t="inlineStr">
+        <is>
+          <t>30%</t>
+        </is>
+      </c>
+      <c r="CE6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="CF6" t="n">
+        <v>30</v>
+      </c>
+      <c r="CG6" t="inlineStr">
+        <is>
+          <t>Equities — UK Large Cap</t>
+        </is>
+      </c>
+      <c r="CH6" t="inlineStr">
+        <is>
+          <t>26%</t>
+        </is>
+      </c>
+      <c r="CI6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="CJ6" t="n">
+        <v>26</v>
+      </c>
+      <c r="CK6" t="inlineStr">
+        <is>
+          <t>Cash &amp; Money Market</t>
+        </is>
+      </c>
+      <c r="CL6" t="inlineStr">
+        <is>
+          <t>14%</t>
+        </is>
+      </c>
+      <c r="CM6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="CN6" t="n">
+        <v>14</v>
+      </c>
+      <c r="CO6" t="inlineStr">
+        <is>
+          <t>Balanced</t>
+        </is>
+      </c>
+      <c r="CP6" t="inlineStr">
+        <is>
+          <t>5–10 years</t>
+        </is>
+      </c>
+      <c r="CQ6" t="inlineStr">
+        <is>
+          <t>Intermediate</t>
+        </is>
+      </c>
+      <c r="CR6" t="inlineStr">
+        <is>
+          <t>2025-11-14</t>
+        </is>
+      </c>
+      <c r="CS6" t="inlineStr">
+        <is>
+          <t>Aligned with Balanced mandate</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -1288,6 +2133,274 @@
           <t>CRD-CH-0231</t>
         </is>
       </c>
+      <c r="AJ7" t="inlineStr">
+        <is>
+          <t>RM</t>
+        </is>
+      </c>
+      <c r="AK7" t="inlineStr">
+        <is>
+          <t>New adverse-media hit — review required</t>
+        </is>
+      </c>
+      <c r="AL7" t="inlineStr">
+        <is>
+          <t>The overnight WorldCheck screen returned a new adverse-media match. Review the identifier comparison and matched article, then confirm a true hit (escalate to Compliance) or dismiss as a false positive.</t>
+        </is>
+      </c>
+      <c r="AM7" t="inlineStr">
+        <is>
+          <t>Review screening hit</t>
+        </is>
+      </c>
+      <c r="AN7" t="inlineStr">
+        <is>
+          <t>cont_screen_CH-priv-0231</t>
+        </is>
+      </c>
+      <c r="AO7" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="AP7" t="inlineStr">
+        <is>
+          <t>WorldCheck (overnight screen)</t>
+        </is>
+      </c>
+      <c r="AQ7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AS7" t="inlineStr">
+        <is>
+          <t>Match</t>
+        </is>
+      </c>
+      <c r="AT7" t="inlineStr">
+        <is>
+          <t>New adverse-media hit — litigation article</t>
+        </is>
+      </c>
+      <c r="AU7" t="inlineStr">
+        <is>
+          <t>danger</t>
+        </is>
+      </c>
+      <c r="AW7" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="AX7" t="inlineStr">
+        <is>
+          <t>Pending RM review — confirm true match</t>
+        </is>
+      </c>
+      <c r="AY7" t="inlineStr">
+        <is>
+          <t>danger</t>
+        </is>
+      </c>
+      <c r="BA7" t="inlineStr">
+        <is>
+          <t>Portfolio return (YTD)</t>
+        </is>
+      </c>
+      <c r="BB7" t="inlineStr">
+        <is>
+          <t>+6.4%</t>
+        </is>
+      </c>
+      <c r="BC7" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="BE7" t="inlineStr">
+        <is>
+          <t>Benchmark — 60/40 blended</t>
+        </is>
+      </c>
+      <c r="BF7" t="inlineStr">
+        <is>
+          <t>+6.1%</t>
+        </is>
+      </c>
+      <c r="BG7" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="BI7" t="inlineStr">
+        <is>
+          <t>Variance vs benchmark</t>
+        </is>
+      </c>
+      <c r="BJ7" t="inlineStr">
+        <is>
+          <t>+0.3 pp</t>
+        </is>
+      </c>
+      <c r="BK7" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="BM7" t="inlineStr">
+        <is>
+          <t>Advisory — Balanced</t>
+        </is>
+      </c>
+      <c r="BN7" t="inlineStr">
+        <is>
+          <t>Equity</t>
+        </is>
+      </c>
+      <c r="BO7" t="inlineStr">
+        <is>
+          <t>55% (ceiling 60%)</t>
+        </is>
+      </c>
+      <c r="BP7" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="BQ7" t="n">
+        <v>55</v>
+      </c>
+      <c r="BR7" t="inlineStr">
+        <is>
+          <t>Fixed income</t>
+        </is>
+      </c>
+      <c r="BS7" t="inlineStr">
+        <is>
+          <t>30% (band ≤45%)</t>
+        </is>
+      </c>
+      <c r="BT7" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="BU7" t="n">
+        <v>30</v>
+      </c>
+      <c r="BV7" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="BW7" t="inlineStr">
+        <is>
+          <t>15% (band ≥5%)</t>
+        </is>
+      </c>
+      <c r="BX7" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="BY7" t="n">
+        <v>15</v>
+      </c>
+      <c r="BZ7" t="inlineStr">
+        <is>
+          <t>Retail — MiFID standard</t>
+        </is>
+      </c>
+      <c r="CA7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CB7" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="CC7" t="inlineStr">
+        <is>
+          <t>Equities — Swiss Large Cap</t>
+        </is>
+      </c>
+      <c r="CD7" t="inlineStr">
+        <is>
+          <t>32%</t>
+        </is>
+      </c>
+      <c r="CE7" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="CF7" t="n">
+        <v>32</v>
+      </c>
+      <c r="CG7" t="inlineStr">
+        <is>
+          <t>Fixed Income — CHF Corporate</t>
+        </is>
+      </c>
+      <c r="CH7" t="inlineStr">
+        <is>
+          <t>28%</t>
+        </is>
+      </c>
+      <c r="CI7" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="CJ7" t="n">
+        <v>28</v>
+      </c>
+      <c r="CK7" t="inlineStr">
+        <is>
+          <t>Real Estate Funds</t>
+        </is>
+      </c>
+      <c r="CL7" t="inlineStr">
+        <is>
+          <t>12%</t>
+        </is>
+      </c>
+      <c r="CM7" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="CN7" t="n">
+        <v>12</v>
+      </c>
+      <c r="CO7" t="inlineStr">
+        <is>
+          <t>Balanced</t>
+        </is>
+      </c>
+      <c r="CP7" t="inlineStr">
+        <is>
+          <t>5–10 years</t>
+        </is>
+      </c>
+      <c r="CQ7" t="inlineStr">
+        <is>
+          <t>Intermediate</t>
+        </is>
+      </c>
+      <c r="CR7" t="inlineStr">
+        <is>
+          <t>2026-01-22</t>
+        </is>
+      </c>
+      <c r="CS7" t="inlineStr">
+        <is>
+          <t>Aligned with Balanced mandate</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
@@ -1459,6 +2572,229 @@
           <t>CRD-CH-0512</t>
         </is>
       </c>
+      <c r="AJ8" t="inlineStr">
+        <is>
+          <t>RM</t>
+        </is>
+      </c>
+      <c r="AK8" t="inlineStr">
+        <is>
+          <t>Allocation breaches risk profile — rebalance</t>
+        </is>
+      </c>
+      <c r="AL8" t="inlineStr">
+        <is>
+          <t>Equity exposure is 72% against a 60% ceiling for a Balanced profile — beyond tolerance, so rebalancing is mandatory. A print-ready rebalancing proposal (trims, redeployment, UK CGT and cost impact, staged execution) is available.</t>
+        </is>
+      </c>
+      <c r="AM8" t="inlineStr">
+        <is>
+          <t>Open rebalancing proposal</t>
+        </is>
+      </c>
+      <c r="AN8" t="inlineStr">
+        <is>
+          <t>cont_reb_REB-2026-Q3-PSH-001</t>
+        </is>
+      </c>
+      <c r="BA8" t="inlineStr">
+        <is>
+          <t>Portfolio return (YTD)</t>
+        </is>
+      </c>
+      <c r="BB8" t="inlineStr">
+        <is>
+          <t>+4.1%</t>
+        </is>
+      </c>
+      <c r="BC8" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="BE8" t="inlineStr">
+        <is>
+          <t>Benchmark — 60/40 blended</t>
+        </is>
+      </c>
+      <c r="BF8" t="inlineStr">
+        <is>
+          <t>+7.8%</t>
+        </is>
+      </c>
+      <c r="BG8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BI8" t="inlineStr">
+        <is>
+          <t>Variance vs benchmark</t>
+        </is>
+      </c>
+      <c r="BJ8" t="inlineStr">
+        <is>
+          <t>-3.7 pp</t>
+        </is>
+      </c>
+      <c r="BK8" t="inlineStr">
+        <is>
+          <t>danger</t>
+        </is>
+      </c>
+      <c r="BM8" t="inlineStr">
+        <is>
+          <t>Discretionary — Balanced Growth</t>
+        </is>
+      </c>
+      <c r="BN8" t="inlineStr">
+        <is>
+          <t>Equity</t>
+        </is>
+      </c>
+      <c r="BO8" t="inlineStr">
+        <is>
+          <t>72% (ceiling 60%)</t>
+        </is>
+      </c>
+      <c r="BP8" t="inlineStr">
+        <is>
+          <t>danger</t>
+        </is>
+      </c>
+      <c r="BQ8" t="n">
+        <v>72</v>
+      </c>
+      <c r="BR8" t="inlineStr">
+        <is>
+          <t>Fixed income</t>
+        </is>
+      </c>
+      <c r="BS8" t="inlineStr">
+        <is>
+          <t>20% (band ≤35%)</t>
+        </is>
+      </c>
+      <c r="BT8" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="BU8" t="n">
+        <v>20</v>
+      </c>
+      <c r="BV8" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="BW8" t="inlineStr">
+        <is>
+          <t>8% (band ≥5%)</t>
+        </is>
+      </c>
+      <c r="BX8" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="BY8" t="n">
+        <v>8</v>
+      </c>
+      <c r="BZ8" t="inlineStr">
+        <is>
+          <t>Retail — MiFID standard</t>
+        </is>
+      </c>
+      <c r="CA8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CB8" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="CC8" t="inlineStr">
+        <is>
+          <t>Equities — Single-name concentration (TechCorp)</t>
+        </is>
+      </c>
+      <c r="CD8" t="inlineStr">
+        <is>
+          <t>22%</t>
+        </is>
+      </c>
+      <c r="CE8" t="inlineStr">
+        <is>
+          <t>warn</t>
+        </is>
+      </c>
+      <c r="CF8" t="n">
+        <v>22</v>
+      </c>
+      <c r="CG8" t="inlineStr">
+        <is>
+          <t>Fixed Income — EM Sovereign</t>
+        </is>
+      </c>
+      <c r="CH8" t="inlineStr">
+        <is>
+          <t>20%</t>
+        </is>
+      </c>
+      <c r="CI8" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="CJ8" t="n">
+        <v>20</v>
+      </c>
+      <c r="CK8" t="inlineStr">
+        <is>
+          <t>Alternatives — Hedge Funds</t>
+        </is>
+      </c>
+      <c r="CL8" t="inlineStr">
+        <is>
+          <t>15%</t>
+        </is>
+      </c>
+      <c r="CM8" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="CN8" t="n">
+        <v>15</v>
+      </c>
+      <c r="CO8" t="inlineStr">
+        <is>
+          <t>Balanced</t>
+        </is>
+      </c>
+      <c r="CP8" t="inlineStr">
+        <is>
+          <t>5–10 years</t>
+        </is>
+      </c>
+      <c r="CQ8" t="inlineStr">
+        <is>
+          <t>Intermediate</t>
+        </is>
+      </c>
+      <c r="CR8" t="inlineStr">
+        <is>
+          <t>2025-09-10</t>
+        </is>
+      </c>
+      <c r="CS8" t="inlineStr">
+        <is>
+          <t>Review needed — allocation drift from mandate</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
@@ -1630,6 +2966,229 @@
           <t>CRD-CH-0658</t>
         </is>
       </c>
+      <c r="AJ9" t="inlineStr">
+        <is>
+          <t>RM</t>
+        </is>
+      </c>
+      <c r="AK9" t="inlineStr">
+        <is>
+          <t>Regulatory change — res non-dom in scope</t>
+        </is>
+      </c>
+      <c r="AL9" t="inlineStr">
+        <is>
+          <t>A new FCA-referenced res non-dom rule (KB-REG-2026-04 v2) uploaded by Compliance to the knowledge base places this UK-resident, Singapore-domiciled client in scope. Complete the impacted-accounts compliance training module.</t>
+        </is>
+      </c>
+      <c r="AM9" t="inlineStr">
+        <is>
+          <t>Go to compliance training</t>
+        </is>
+      </c>
+      <c r="AN9" t="inlineStr">
+        <is>
+          <t>https://example.com/compliance/training/KB-REG-2026-04</t>
+        </is>
+      </c>
+      <c r="BA9" t="inlineStr">
+        <is>
+          <t>Portfolio return (YTD)</t>
+        </is>
+      </c>
+      <c r="BB9" t="inlineStr">
+        <is>
+          <t>+8.9%</t>
+        </is>
+      </c>
+      <c r="BC9" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="BE9" t="inlineStr">
+        <is>
+          <t>Benchmark — MSCI ACWI</t>
+        </is>
+      </c>
+      <c r="BF9" t="inlineStr">
+        <is>
+          <t>+8.4%</t>
+        </is>
+      </c>
+      <c r="BG9" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="BI9" t="inlineStr">
+        <is>
+          <t>Variance vs benchmark</t>
+        </is>
+      </c>
+      <c r="BJ9" t="inlineStr">
+        <is>
+          <t>+0.5 pp</t>
+        </is>
+      </c>
+      <c r="BK9" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="BM9" t="inlineStr">
+        <is>
+          <t>Discretionary — Growth</t>
+        </is>
+      </c>
+      <c r="BN9" t="inlineStr">
+        <is>
+          <t>Equity</t>
+        </is>
+      </c>
+      <c r="BO9" t="inlineStr">
+        <is>
+          <t>68% (ceiling 75%)</t>
+        </is>
+      </c>
+      <c r="BP9" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="BQ9" t="n">
+        <v>68</v>
+      </c>
+      <c r="BR9" t="inlineStr">
+        <is>
+          <t>Fixed income</t>
+        </is>
+      </c>
+      <c r="BS9" t="inlineStr">
+        <is>
+          <t>20% (band ≤30%)</t>
+        </is>
+      </c>
+      <c r="BT9" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="BU9" t="n">
+        <v>20</v>
+      </c>
+      <c r="BV9" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="BW9" t="inlineStr">
+        <is>
+          <t>12% (band ≥5%)</t>
+        </is>
+      </c>
+      <c r="BX9" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="BY9" t="n">
+        <v>12</v>
+      </c>
+      <c r="BZ9" t="inlineStr">
+        <is>
+          <t>Retail</t>
+        </is>
+      </c>
+      <c r="CA9" t="inlineStr">
+        <is>
+          <t>Elective-professional</t>
+        </is>
+      </c>
+      <c r="CB9" t="inlineStr">
+        <is>
+          <t>Rule KB-REG-2026-04 v2 (FCA) — reassessment required</t>
+        </is>
+      </c>
+      <c r="CC9" t="inlineStr">
+        <is>
+          <t>Equities — Non-dom offshore structures</t>
+        </is>
+      </c>
+      <c r="CD9" t="inlineStr">
+        <is>
+          <t>30%</t>
+        </is>
+      </c>
+      <c r="CE9" t="inlineStr">
+        <is>
+          <t>warn</t>
+        </is>
+      </c>
+      <c r="CF9" t="n">
+        <v>30</v>
+      </c>
+      <c r="CG9" t="inlineStr">
+        <is>
+          <t>Fixed Income — Global Aggregate</t>
+        </is>
+      </c>
+      <c r="CH9" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="CI9" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="CJ9" t="n">
+        <v>25</v>
+      </c>
+      <c r="CK9" t="inlineStr">
+        <is>
+          <t>Cash &amp; Money Market</t>
+        </is>
+      </c>
+      <c r="CL9" t="inlineStr">
+        <is>
+          <t>12%</t>
+        </is>
+      </c>
+      <c r="CM9" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="CN9" t="n">
+        <v>12</v>
+      </c>
+      <c r="CO9" t="inlineStr">
+        <is>
+          <t>Growth</t>
+        </is>
+      </c>
+      <c r="CP9" t="inlineStr">
+        <is>
+          <t>10+ years</t>
+        </is>
+      </c>
+      <c r="CQ9" t="inlineStr">
+        <is>
+          <t>Advanced</t>
+        </is>
+      </c>
+      <c r="CR9" t="inlineStr">
+        <is>
+          <t>2025-12-01</t>
+        </is>
+      </c>
+      <c r="CS9" t="inlineStr">
+        <is>
+          <t>Aligned with Growth mandate</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
@@ -1801,6 +3360,274 @@
           <t>CRD-CH-0847</t>
         </is>
       </c>
+      <c r="AJ10" t="inlineStr">
+        <is>
+          <t>RM</t>
+        </is>
+      </c>
+      <c r="AK10" t="inlineStr">
+        <is>
+          <t>Passport expiring — request renewal</t>
+        </is>
+      </c>
+      <c r="AL10" t="inlineStr">
+        <is>
+          <t>The client's passport expires on 2026-08-03. Triggered ahead of expiry: draft an Outlook email requesting a certified copy of the renewed passport. The draft lands in Drafts for the RM to review and send — never auto-sent.</t>
+        </is>
+      </c>
+      <c r="AM10" t="inlineStr">
+        <is>
+          <t>Draft email in Outlook</t>
+        </is>
+      </c>
+      <c r="AN10" t="inlineStr">
+        <is>
+          <t>cont_outlook_draft_CH-priv-0847</t>
+        </is>
+      </c>
+      <c r="AO10" t="inlineStr">
+        <is>
+          <t>Passport</t>
+        </is>
+      </c>
+      <c r="AP10" t="inlineStr">
+        <is>
+          <t>Expires 2026-08-03 (13 days)</t>
+        </is>
+      </c>
+      <c r="AQ10" t="inlineStr">
+        <is>
+          <t>danger</t>
+        </is>
+      </c>
+      <c r="AS10" t="inlineStr">
+        <is>
+          <t>Proof of address</t>
+        </is>
+      </c>
+      <c r="AT10" t="inlineStr">
+        <is>
+          <t>On file — valid</t>
+        </is>
+      </c>
+      <c r="AU10" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="AW10" t="inlineStr">
+        <is>
+          <t>Periodic KYC refresh</t>
+        </is>
+      </c>
+      <c r="AX10" t="inlineStr">
+        <is>
+          <t>Completed 2024 · next due 2027</t>
+        </is>
+      </c>
+      <c r="AY10" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="BA10" t="inlineStr">
+        <is>
+          <t>Portfolio return (YTD)</t>
+        </is>
+      </c>
+      <c r="BB10" t="inlineStr">
+        <is>
+          <t>+3.1%</t>
+        </is>
+      </c>
+      <c r="BC10" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="BE10" t="inlineStr">
+        <is>
+          <t>Benchmark — 20/80 blended</t>
+        </is>
+      </c>
+      <c r="BF10" t="inlineStr">
+        <is>
+          <t>+3.4%</t>
+        </is>
+      </c>
+      <c r="BG10" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="BI10" t="inlineStr">
+        <is>
+          <t>Variance vs benchmark</t>
+        </is>
+      </c>
+      <c r="BJ10" t="inlineStr">
+        <is>
+          <t>-0.3 pp</t>
+        </is>
+      </c>
+      <c r="BK10" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="BM10" t="inlineStr">
+        <is>
+          <t>Advisory — Conservative</t>
+        </is>
+      </c>
+      <c r="BN10" t="inlineStr">
+        <is>
+          <t>Equity</t>
+        </is>
+      </c>
+      <c r="BO10" t="inlineStr">
+        <is>
+          <t>28% (ceiling 40%)</t>
+        </is>
+      </c>
+      <c r="BP10" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="BQ10" t="n">
+        <v>28</v>
+      </c>
+      <c r="BR10" t="inlineStr">
+        <is>
+          <t>Fixed income</t>
+        </is>
+      </c>
+      <c r="BS10" t="inlineStr">
+        <is>
+          <t>58% (band ≤65%)</t>
+        </is>
+      </c>
+      <c r="BT10" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="BU10" t="n">
+        <v>58</v>
+      </c>
+      <c r="BV10" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="BW10" t="inlineStr">
+        <is>
+          <t>14% (band ≥10%)</t>
+        </is>
+      </c>
+      <c r="BX10" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="BY10" t="n">
+        <v>14</v>
+      </c>
+      <c r="BZ10" t="inlineStr">
+        <is>
+          <t>Retail — MiFID standard</t>
+        </is>
+      </c>
+      <c r="CA10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CB10" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="CC10" t="inlineStr">
+        <is>
+          <t>Fixed Income — CHF Government</t>
+        </is>
+      </c>
+      <c r="CD10" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="CE10" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="CF10" t="n">
+        <v>40</v>
+      </c>
+      <c r="CG10" t="inlineStr">
+        <is>
+          <t>Fixed Income — IG Corporate</t>
+        </is>
+      </c>
+      <c r="CH10" t="inlineStr">
+        <is>
+          <t>22%</t>
+        </is>
+      </c>
+      <c r="CI10" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="CJ10" t="n">
+        <v>22</v>
+      </c>
+      <c r="CK10" t="inlineStr">
+        <is>
+          <t>Cash &amp; Money Market</t>
+        </is>
+      </c>
+      <c r="CL10" t="inlineStr">
+        <is>
+          <t>14%</t>
+        </is>
+      </c>
+      <c r="CM10" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="CN10" t="n">
+        <v>14</v>
+      </c>
+      <c r="CO10" t="inlineStr">
+        <is>
+          <t>Conservative</t>
+        </is>
+      </c>
+      <c r="CP10" t="inlineStr">
+        <is>
+          <t>3–5 years</t>
+        </is>
+      </c>
+      <c r="CQ10" t="inlineStr">
+        <is>
+          <t>Basic</t>
+        </is>
+      </c>
+      <c r="CR10" t="inlineStr">
+        <is>
+          <t>2026-02-18</t>
+        </is>
+      </c>
+      <c r="CS10" t="inlineStr">
+        <is>
+          <t>Aligned with Conservative mandate</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
@@ -1972,6 +3799,229 @@
           <t>CRD-CH-0093</t>
         </is>
       </c>
+      <c r="AJ11" t="inlineStr">
+        <is>
+          <t>RM</t>
+        </is>
+      </c>
+      <c r="AK11" t="inlineStr">
+        <is>
+          <t>Suitability review due</t>
+        </is>
+      </c>
+      <c r="AL11" t="inlineStr">
+        <is>
+          <t>The annual suitability review is due. Complete the questionnaire, prefilled from CRM (email fallback if prefill is unavailable).</t>
+        </is>
+      </c>
+      <c r="AM11" t="inlineStr">
+        <is>
+          <t>Complete questionnaire</t>
+        </is>
+      </c>
+      <c r="AN11" t="inlineStr">
+        <is>
+          <t>cont_suit_CH-priv-0093</t>
+        </is>
+      </c>
+      <c r="BA11" t="inlineStr">
+        <is>
+          <t>Portfolio return (YTD)</t>
+        </is>
+      </c>
+      <c r="BB11" t="inlineStr">
+        <is>
+          <t>+5.9%</t>
+        </is>
+      </c>
+      <c r="BC11" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="BE11" t="inlineStr">
+        <is>
+          <t>Benchmark — 60/40 blended</t>
+        </is>
+      </c>
+      <c r="BF11" t="inlineStr">
+        <is>
+          <t>+6.1%</t>
+        </is>
+      </c>
+      <c r="BG11" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="BI11" t="inlineStr">
+        <is>
+          <t>Variance vs benchmark</t>
+        </is>
+      </c>
+      <c r="BJ11" t="inlineStr">
+        <is>
+          <t>-0.2 pp</t>
+        </is>
+      </c>
+      <c r="BK11" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="BM11" t="inlineStr">
+        <is>
+          <t>Discretionary — Balanced</t>
+        </is>
+      </c>
+      <c r="BN11" t="inlineStr">
+        <is>
+          <t>Equity</t>
+        </is>
+      </c>
+      <c r="BO11" t="inlineStr">
+        <is>
+          <t>50% (ceiling 60%)</t>
+        </is>
+      </c>
+      <c r="BP11" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="BQ11" t="n">
+        <v>50</v>
+      </c>
+      <c r="BR11" t="inlineStr">
+        <is>
+          <t>Fixed income</t>
+        </is>
+      </c>
+      <c r="BS11" t="inlineStr">
+        <is>
+          <t>36% (band ≤45%)</t>
+        </is>
+      </c>
+      <c r="BT11" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="BU11" t="n">
+        <v>36</v>
+      </c>
+      <c r="BV11" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="BW11" t="inlineStr">
+        <is>
+          <t>14% (band ≥5%)</t>
+        </is>
+      </c>
+      <c r="BX11" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="BY11" t="n">
+        <v>14</v>
+      </c>
+      <c r="BZ11" t="inlineStr">
+        <is>
+          <t>Retail — MiFID standard</t>
+        </is>
+      </c>
+      <c r="CA11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CB11" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="CC11" t="inlineStr">
+        <is>
+          <t>Equities — European Large Cap</t>
+        </is>
+      </c>
+      <c r="CD11" t="inlineStr">
+        <is>
+          <t>28%</t>
+        </is>
+      </c>
+      <c r="CE11" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="CF11" t="n">
+        <v>28</v>
+      </c>
+      <c r="CG11" t="inlineStr">
+        <is>
+          <t>Fixed Income — EUR Corporate</t>
+        </is>
+      </c>
+      <c r="CH11" t="inlineStr">
+        <is>
+          <t>26%</t>
+        </is>
+      </c>
+      <c r="CI11" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="CJ11" t="n">
+        <v>26</v>
+      </c>
+      <c r="CK11" t="inlineStr">
+        <is>
+          <t>Multi-Asset Funds</t>
+        </is>
+      </c>
+      <c r="CL11" t="inlineStr">
+        <is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="CM11" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="CN11" t="n">
+        <v>16</v>
+      </c>
+      <c r="CO11" t="inlineStr">
+        <is>
+          <t>Balanced</t>
+        </is>
+      </c>
+      <c r="CP11" t="inlineStr">
+        <is>
+          <t>5–10 years</t>
+        </is>
+      </c>
+      <c r="CQ11" t="inlineStr">
+        <is>
+          <t>Intermediate</t>
+        </is>
+      </c>
+      <c r="CR11" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="CS11" t="inlineStr">
+        <is>
+          <t>Annual review due — ongoing, needs-based cadence</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
@@ -2141,6 +4191,274 @@
       <c r="AI12" t="inlineStr">
         <is>
           <t>CRD-CH-0774</t>
+        </is>
+      </c>
+      <c r="AJ12" t="inlineStr">
+        <is>
+          <t>RM</t>
+        </is>
+      </c>
+      <c r="AK12" t="inlineStr">
+        <is>
+          <t>Source-of-wealth refresh</t>
+        </is>
+      </c>
+      <c r="AL12" t="inlineStr">
+        <is>
+          <t>An incoming transfer of CHF 2,400,000 is not covered by the source-of-wealth narrative on file. Launch the SoW Agent to re-assess and corroborate the new wealth event (D&amp;B ownership records, documents on file).</t>
+        </is>
+      </c>
+      <c r="AM12" t="inlineStr">
+        <is>
+          <t>Launch SoW assessment</t>
+        </is>
+      </c>
+      <c r="AN12" t="inlineStr">
+        <is>
+          <t>cont_sow_CH-priv-0774</t>
+        </is>
+      </c>
+      <c r="AO12" t="inlineStr">
+        <is>
+          <t>Incoming transfer</t>
+        </is>
+      </c>
+      <c r="AP12" t="inlineStr">
+        <is>
+          <t>CHF 2,400,000 (18 Jul)</t>
+        </is>
+      </c>
+      <c r="AQ12" t="inlineStr">
+        <is>
+          <t>warn</t>
+        </is>
+      </c>
+      <c r="AS12" t="inlineStr">
+        <is>
+          <t>Narrative on file</t>
+        </is>
+      </c>
+      <c r="AT12" t="inlineStr">
+        <is>
+          <t>Does not cover this event</t>
+        </is>
+      </c>
+      <c r="AU12" t="inlineStr">
+        <is>
+          <t>danger</t>
+        </is>
+      </c>
+      <c r="AW12" t="inlineStr">
+        <is>
+          <t>Suggested evidence</t>
+        </is>
+      </c>
+      <c r="AX12" t="inlineStr">
+        <is>
+          <t>Company sale agreement</t>
+        </is>
+      </c>
+      <c r="AY12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BA12" t="inlineStr">
+        <is>
+          <t>Portfolio return (YTD)</t>
+        </is>
+      </c>
+      <c r="BB12" t="inlineStr">
+        <is>
+          <t>+10.1%</t>
+        </is>
+      </c>
+      <c r="BC12" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="BE12" t="inlineStr">
+        <is>
+          <t>Benchmark — MSCI ACWI</t>
+        </is>
+      </c>
+      <c r="BF12" t="inlineStr">
+        <is>
+          <t>+8.4%</t>
+        </is>
+      </c>
+      <c r="BG12" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="BI12" t="inlineStr">
+        <is>
+          <t>Variance vs benchmark</t>
+        </is>
+      </c>
+      <c r="BJ12" t="inlineStr">
+        <is>
+          <t>+1.7 pp</t>
+        </is>
+      </c>
+      <c r="BK12" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="BM12" t="inlineStr">
+        <is>
+          <t>Discretionary — Growth</t>
+        </is>
+      </c>
+      <c r="BN12" t="inlineStr">
+        <is>
+          <t>Equity</t>
+        </is>
+      </c>
+      <c r="BO12" t="inlineStr">
+        <is>
+          <t>70% (ceiling 75%)</t>
+        </is>
+      </c>
+      <c r="BP12" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="BQ12" t="n">
+        <v>70</v>
+      </c>
+      <c r="BR12" t="inlineStr">
+        <is>
+          <t>Fixed income</t>
+        </is>
+      </c>
+      <c r="BS12" t="inlineStr">
+        <is>
+          <t>20% (band ≤30%)</t>
+        </is>
+      </c>
+      <c r="BT12" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="BU12" t="n">
+        <v>20</v>
+      </c>
+      <c r="BV12" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="BW12" t="inlineStr">
+        <is>
+          <t>10% (band ≥5%)</t>
+        </is>
+      </c>
+      <c r="BX12" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="BY12" t="n">
+        <v>10</v>
+      </c>
+      <c r="BZ12" t="inlineStr">
+        <is>
+          <t>Professional client (per-se)</t>
+        </is>
+      </c>
+      <c r="CA12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CB12" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="CC12" t="inlineStr">
+        <is>
+          <t>Equities — Global Large Cap</t>
+        </is>
+      </c>
+      <c r="CD12" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="CE12" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="CF12" t="n">
+        <v>40</v>
+      </c>
+      <c r="CG12" t="inlineStr">
+        <is>
+          <t>Private Equity</t>
+        </is>
+      </c>
+      <c r="CH12" t="inlineStr">
+        <is>
+          <t>22%</t>
+        </is>
+      </c>
+      <c r="CI12" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="CJ12" t="n">
+        <v>22</v>
+      </c>
+      <c r="CK12" t="inlineStr">
+        <is>
+          <t>Cash &amp; Money Market</t>
+        </is>
+      </c>
+      <c r="CL12" t="inlineStr">
+        <is>
+          <t>10%</t>
+        </is>
+      </c>
+      <c r="CM12" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="CN12" t="n">
+        <v>10</v>
+      </c>
+      <c r="CO12" t="inlineStr">
+        <is>
+          <t>Growth</t>
+        </is>
+      </c>
+      <c r="CP12" t="inlineStr">
+        <is>
+          <t>10+ years</t>
+        </is>
+      </c>
+      <c r="CQ12" t="inlineStr">
+        <is>
+          <t>Advanced</t>
+        </is>
+      </c>
+      <c r="CR12" t="inlineStr">
+        <is>
+          <t>2025-10-05</t>
+        </is>
+      </c>
+      <c r="CS12" t="inlineStr">
+        <is>
+          <t>Aligned with Growth mandate</t>
         </is>
       </c>
     </row>
@@ -2280,6 +4598,204 @@
           <t>CRD-CH-0901</t>
         </is>
       </c>
+      <c r="BA13" t="inlineStr">
+        <is>
+          <t>Portfolio return (YTD)</t>
+        </is>
+      </c>
+      <c r="BB13" t="inlineStr">
+        <is>
+          <t>+6.0%</t>
+        </is>
+      </c>
+      <c r="BC13" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="BE13" t="inlineStr">
+        <is>
+          <t>Benchmark — 60/40 blended</t>
+        </is>
+      </c>
+      <c r="BF13" t="inlineStr">
+        <is>
+          <t>+6.1%</t>
+        </is>
+      </c>
+      <c r="BG13" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="BI13" t="inlineStr">
+        <is>
+          <t>Variance vs benchmark</t>
+        </is>
+      </c>
+      <c r="BJ13" t="inlineStr">
+        <is>
+          <t>-0.1 pp</t>
+        </is>
+      </c>
+      <c r="BK13" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="BM13" t="inlineStr">
+        <is>
+          <t>Advisory — Balanced</t>
+        </is>
+      </c>
+      <c r="BN13" t="inlineStr">
+        <is>
+          <t>Equity</t>
+        </is>
+      </c>
+      <c r="BO13" t="inlineStr">
+        <is>
+          <t>52% (ceiling 60%)</t>
+        </is>
+      </c>
+      <c r="BP13" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="BQ13" t="n">
+        <v>52</v>
+      </c>
+      <c r="BR13" t="inlineStr">
+        <is>
+          <t>Fixed income</t>
+        </is>
+      </c>
+      <c r="BS13" t="inlineStr">
+        <is>
+          <t>34% (band ≤45%)</t>
+        </is>
+      </c>
+      <c r="BT13" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="BU13" t="n">
+        <v>34</v>
+      </c>
+      <c r="BV13" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="BW13" t="inlineStr">
+        <is>
+          <t>14% (band ≥5%)</t>
+        </is>
+      </c>
+      <c r="BX13" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="BY13" t="n">
+        <v>14</v>
+      </c>
+      <c r="BZ13" t="inlineStr">
+        <is>
+          <t>Professional client (per-se)</t>
+        </is>
+      </c>
+      <c r="CA13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CB13" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="CC13" t="inlineStr">
+        <is>
+          <t>Equities — Eurozone Large Cap</t>
+        </is>
+      </c>
+      <c r="CD13" t="inlineStr">
+        <is>
+          <t>30%</t>
+        </is>
+      </c>
+      <c r="CE13" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="CF13" t="n">
+        <v>30</v>
+      </c>
+      <c r="CG13" t="inlineStr">
+        <is>
+          <t>Fixed Income — EUR Government</t>
+        </is>
+      </c>
+      <c r="CH13" t="inlineStr">
+        <is>
+          <t>28%</t>
+        </is>
+      </c>
+      <c r="CI13" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="CJ13" t="n">
+        <v>28</v>
+      </c>
+      <c r="CK13" t="inlineStr">
+        <is>
+          <t>Cash &amp; Money Market</t>
+        </is>
+      </c>
+      <c r="CL13" t="inlineStr">
+        <is>
+          <t>14%</t>
+        </is>
+      </c>
+      <c r="CM13" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="CN13" t="n">
+        <v>14</v>
+      </c>
+      <c r="CO13" t="inlineStr">
+        <is>
+          <t>Balanced</t>
+        </is>
+      </c>
+      <c r="CP13" t="inlineStr">
+        <is>
+          <t>5–10 years</t>
+        </is>
+      </c>
+      <c r="CQ13" t="inlineStr">
+        <is>
+          <t>Advanced — corporate treasury</t>
+        </is>
+      </c>
+      <c r="CR13" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="CS13" t="inlineStr">
+        <is>
+          <t>Aligned with Balanced mandate</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
@@ -2417,6 +4933,204 @@
           <t>CRD-CH-0902</t>
         </is>
       </c>
+      <c r="BA14" t="inlineStr">
+        <is>
+          <t>Portfolio return (YTD)</t>
+        </is>
+      </c>
+      <c r="BB14" t="inlineStr">
+        <is>
+          <t>+2.8%</t>
+        </is>
+      </c>
+      <c r="BC14" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="BE14" t="inlineStr">
+        <is>
+          <t>Benchmark — 20/80 blended</t>
+        </is>
+      </c>
+      <c r="BF14" t="inlineStr">
+        <is>
+          <t>+3.4%</t>
+        </is>
+      </c>
+      <c r="BG14" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="BI14" t="inlineStr">
+        <is>
+          <t>Variance vs benchmark</t>
+        </is>
+      </c>
+      <c r="BJ14" t="inlineStr">
+        <is>
+          <t>-0.6 pp</t>
+        </is>
+      </c>
+      <c r="BK14" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="BM14" t="inlineStr">
+        <is>
+          <t>Advisory — Conservative</t>
+        </is>
+      </c>
+      <c r="BN14" t="inlineStr">
+        <is>
+          <t>Equity</t>
+        </is>
+      </c>
+      <c r="BO14" t="inlineStr">
+        <is>
+          <t>25% (ceiling 40%)</t>
+        </is>
+      </c>
+      <c r="BP14" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="BQ14" t="n">
+        <v>25</v>
+      </c>
+      <c r="BR14" t="inlineStr">
+        <is>
+          <t>Fixed income</t>
+        </is>
+      </c>
+      <c r="BS14" t="inlineStr">
+        <is>
+          <t>60% (band ≤65%)</t>
+        </is>
+      </c>
+      <c r="BT14" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="BU14" t="n">
+        <v>60</v>
+      </c>
+      <c r="BV14" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="BW14" t="inlineStr">
+        <is>
+          <t>15% (band ≥10%)</t>
+        </is>
+      </c>
+      <c r="BX14" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="BY14" t="n">
+        <v>15</v>
+      </c>
+      <c r="BZ14" t="inlineStr">
+        <is>
+          <t>Professional client (per-se)</t>
+        </is>
+      </c>
+      <c r="CA14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CB14" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="CC14" t="inlineStr">
+        <is>
+          <t>Fixed Income — JGB</t>
+        </is>
+      </c>
+      <c r="CD14" t="inlineStr">
+        <is>
+          <t>42%</t>
+        </is>
+      </c>
+      <c r="CE14" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="CF14" t="n">
+        <v>42</v>
+      </c>
+      <c r="CG14" t="inlineStr">
+        <is>
+          <t>Fixed Income — Global Aggregate</t>
+        </is>
+      </c>
+      <c r="CH14" t="inlineStr">
+        <is>
+          <t>20%</t>
+        </is>
+      </c>
+      <c r="CI14" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="CJ14" t="n">
+        <v>20</v>
+      </c>
+      <c r="CK14" t="inlineStr">
+        <is>
+          <t>Cash &amp; Money Market</t>
+        </is>
+      </c>
+      <c r="CL14" t="inlineStr">
+        <is>
+          <t>15%</t>
+        </is>
+      </c>
+      <c r="CM14" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="CN14" t="n">
+        <v>15</v>
+      </c>
+      <c r="CO14" t="inlineStr">
+        <is>
+          <t>Conservative</t>
+        </is>
+      </c>
+      <c r="CP14" t="inlineStr">
+        <is>
+          <t>3–5 years</t>
+        </is>
+      </c>
+      <c r="CQ14" t="inlineStr">
+        <is>
+          <t>Intermediate — corporate treasury</t>
+        </is>
+      </c>
+      <c r="CR14" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="CS14" t="inlineStr">
+        <is>
+          <t>Aligned with Conservative mandate</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
@@ -2554,6 +5268,204 @@
           <t>CRD-CH-0903</t>
         </is>
       </c>
+      <c r="BA15" t="inlineStr">
+        <is>
+          <t>Portfolio return (YTD)</t>
+        </is>
+      </c>
+      <c r="BB15" t="inlineStr">
+        <is>
+          <t>+11.4%</t>
+        </is>
+      </c>
+      <c r="BC15" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="BE15" t="inlineStr">
+        <is>
+          <t>Benchmark — MSCI ACWI</t>
+        </is>
+      </c>
+      <c r="BF15" t="inlineStr">
+        <is>
+          <t>+8.4%</t>
+        </is>
+      </c>
+      <c r="BG15" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="BI15" t="inlineStr">
+        <is>
+          <t>Variance vs benchmark</t>
+        </is>
+      </c>
+      <c r="BJ15" t="inlineStr">
+        <is>
+          <t>+3.0 pp</t>
+        </is>
+      </c>
+      <c r="BK15" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="BM15" t="inlineStr">
+        <is>
+          <t>Discretionary — Growth</t>
+        </is>
+      </c>
+      <c r="BN15" t="inlineStr">
+        <is>
+          <t>Equity</t>
+        </is>
+      </c>
+      <c r="BO15" t="inlineStr">
+        <is>
+          <t>72% (ceiling 75%)</t>
+        </is>
+      </c>
+      <c r="BP15" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="BQ15" t="n">
+        <v>72</v>
+      </c>
+      <c r="BR15" t="inlineStr">
+        <is>
+          <t>Fixed income</t>
+        </is>
+      </c>
+      <c r="BS15" t="inlineStr">
+        <is>
+          <t>18% (band ≤30%)</t>
+        </is>
+      </c>
+      <c r="BT15" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="BU15" t="n">
+        <v>18</v>
+      </c>
+      <c r="BV15" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="BW15" t="inlineStr">
+        <is>
+          <t>10% (band ≥5%)</t>
+        </is>
+      </c>
+      <c r="BX15" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="BY15" t="n">
+        <v>10</v>
+      </c>
+      <c r="BZ15" t="inlineStr">
+        <is>
+          <t>Professional client (per-se)</t>
+        </is>
+      </c>
+      <c r="CA15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CB15" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="CC15" t="inlineStr">
+        <is>
+          <t>Equities — Global Large Cap</t>
+        </is>
+      </c>
+      <c r="CD15" t="inlineStr">
+        <is>
+          <t>44%</t>
+        </is>
+      </c>
+      <c r="CE15" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="CF15" t="n">
+        <v>44</v>
+      </c>
+      <c r="CG15" t="inlineStr">
+        <is>
+          <t>Private Equity</t>
+        </is>
+      </c>
+      <c r="CH15" t="inlineStr">
+        <is>
+          <t>20%</t>
+        </is>
+      </c>
+      <c r="CI15" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="CJ15" t="n">
+        <v>20</v>
+      </c>
+      <c r="CK15" t="inlineStr">
+        <is>
+          <t>Cash &amp; Money Market</t>
+        </is>
+      </c>
+      <c r="CL15" t="inlineStr">
+        <is>
+          <t>10%</t>
+        </is>
+      </c>
+      <c r="CM15" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="CN15" t="n">
+        <v>10</v>
+      </c>
+      <c r="CO15" t="inlineStr">
+        <is>
+          <t>Growth</t>
+        </is>
+      </c>
+      <c r="CP15" t="inlineStr">
+        <is>
+          <t>10+ years</t>
+        </is>
+      </c>
+      <c r="CQ15" t="inlineStr">
+        <is>
+          <t>Advanced — corporate treasury</t>
+        </is>
+      </c>
+      <c r="CR15" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="CS15" t="inlineStr">
+        <is>
+          <t>Aligned with Growth mandate</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
@@ -2707,6 +5619,204 @@
       <c r="AI16" t="inlineStr">
         <is>
           <t>CRD-CH-0355</t>
+        </is>
+      </c>
+      <c r="BA16" t="inlineStr">
+        <is>
+          <t>Portfolio return (YTD)</t>
+        </is>
+      </c>
+      <c r="BB16" t="inlineStr">
+        <is>
+          <t>+2.5%</t>
+        </is>
+      </c>
+      <c r="BC16" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="BE16" t="inlineStr">
+        <is>
+          <t>Benchmark — 20/80 blended</t>
+        </is>
+      </c>
+      <c r="BF16" t="inlineStr">
+        <is>
+          <t>+3.4%</t>
+        </is>
+      </c>
+      <c r="BG16" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="BI16" t="inlineStr">
+        <is>
+          <t>Variance vs benchmark</t>
+        </is>
+      </c>
+      <c r="BJ16" t="inlineStr">
+        <is>
+          <t>-0.9 pp</t>
+        </is>
+      </c>
+      <c r="BK16" t="inlineStr">
+        <is>
+          <t>warn</t>
+        </is>
+      </c>
+      <c r="BM16" t="inlineStr">
+        <is>
+          <t>Advisory — Conservative</t>
+        </is>
+      </c>
+      <c r="BN16" t="inlineStr">
+        <is>
+          <t>Equity</t>
+        </is>
+      </c>
+      <c r="BO16" t="inlineStr">
+        <is>
+          <t>22% (ceiling 40%)</t>
+        </is>
+      </c>
+      <c r="BP16" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="BQ16" t="n">
+        <v>22</v>
+      </c>
+      <c r="BR16" t="inlineStr">
+        <is>
+          <t>Fixed income</t>
+        </is>
+      </c>
+      <c r="BS16" t="inlineStr">
+        <is>
+          <t>62% (band ≤65%)</t>
+        </is>
+      </c>
+      <c r="BT16" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="BU16" t="n">
+        <v>62</v>
+      </c>
+      <c r="BV16" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="BW16" t="inlineStr">
+        <is>
+          <t>16% (band ≥10%)</t>
+        </is>
+      </c>
+      <c r="BX16" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="BY16" t="n">
+        <v>16</v>
+      </c>
+      <c r="BZ16" t="inlineStr">
+        <is>
+          <t>Retail — MiFID standard</t>
+        </is>
+      </c>
+      <c r="CA16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="CB16" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="CC16" t="inlineStr">
+        <is>
+          <t>Fixed Income — CHF Government</t>
+        </is>
+      </c>
+      <c r="CD16" t="inlineStr">
+        <is>
+          <t>45%</t>
+        </is>
+      </c>
+      <c r="CE16" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="CF16" t="n">
+        <v>45</v>
+      </c>
+      <c r="CG16" t="inlineStr">
+        <is>
+          <t>Fixed Income — IG Corporate</t>
+        </is>
+      </c>
+      <c r="CH16" t="inlineStr">
+        <is>
+          <t>20%</t>
+        </is>
+      </c>
+      <c r="CI16" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="CJ16" t="n">
+        <v>20</v>
+      </c>
+      <c r="CK16" t="inlineStr">
+        <is>
+          <t>Cash &amp; Money Market</t>
+        </is>
+      </c>
+      <c r="CL16" t="inlineStr">
+        <is>
+          <t>16%</t>
+        </is>
+      </c>
+      <c r="CM16" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="CN16" t="n">
+        <v>16</v>
+      </c>
+      <c r="CO16" t="inlineStr">
+        <is>
+          <t>Conservative</t>
+        </is>
+      </c>
+      <c r="CP16" t="inlineStr">
+        <is>
+          <t>3–5 years</t>
+        </is>
+      </c>
+      <c r="CQ16" t="inlineStr">
+        <is>
+          <t>Basic</t>
+        </is>
+      </c>
+      <c r="CR16" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="CS16" t="inlineStr">
+        <is>
+          <t>Aligned with Conservative mandate</t>
         </is>
       </c>
     </row>
@@ -3499,7 +6609,6 @@
         </is>
       </c>
     </row>
-    <row r="19"/>
     <row r="20">
       <c r="A20" s="15" t="inlineStr">
         <is>
@@ -3591,7 +6700,6 @@
         </is>
       </c>
     </row>
-    <row r="28"/>
     <row r="29">
       <c r="A29" s="15" t="inlineStr">
         <is>

</xml_diff>